<commit_message>
feat: add weapon configs and debug UI
</commit_message>
<xml_diff>
--- a/Config/Excel/DT_StatusEffectConfig.xlsx
+++ b/Config/Excel/DT_StatusEffectConfig.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\UnrealDeepRock_Config_Preview\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7EF307E7-C538-43EB-B77D-6195E8D3533E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1489919-786A-4A87-90B7-B5D2EB8080A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3900" yWindow="3900" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
   <si>
     <t>#TABLE=DT_StatusEffectConfig</t>
   </si>
@@ -134,54 +134,103 @@
   </si>
   <si>
     <t>Burning</t>
-  </si>
-  <si>
-    <t>火焰元素异常</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>火焰喷射器叠层燃烧</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>灼烧</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Status.Burning</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>RefreshDuration</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Frozen</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>冰冻元素异常</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>冰冻</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Status.Frozen</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Shocked</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>电击元素异常</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>感电</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Status.Shocked</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Corroded</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>酸液元素异常</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>腐蚀</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Status.Corroded</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vulnerable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>奥术连弩命中叠加易伤</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>易伤</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Status.Vulnerable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bleeding</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>链锯命中叠加流血</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>流血</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Status.Bleeding</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -528,7 +577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.15">
@@ -697,7 +746,7 @@
         <v>1</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -709,7 +758,7 @@
         <v>0</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N5" t="s">
         <v>41</v>
@@ -835,6 +884,88 @@
         <v>1</v>
       </c>
       <c r="N8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.15">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9">
+        <v>5</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0.05</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>10</v>
+      </c>
+      <c r="N9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.15">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" t="s">
+        <v>61</v>
+      </c>
+      <c r="F10">
+        <v>6</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>4</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>5</v>
+      </c>
+      <c r="N10" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement weapon status effect system
</commit_message>
<xml_diff>
--- a/Config/Excel/DT_StatusEffectConfig.xlsx
+++ b/Config/Excel/DT_StatusEffectConfig.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\testfiles\UnrealDeepRock\LetsDeepRock\Config\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1489919-786A-4A87-90B7-B5D2EB8080A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7D28CA1-BC8A-4BB7-A5C2-AD8835314CF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="3900" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="66">
   <si>
     <t>#TABLE=DT_StatusEffectConfig</t>
   </si>
@@ -231,6 +231,18 @@
   <si>
     <t>Status.Bleeding</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ApplyChance</t>
+  </si>
+  <si>
+    <t>HitsPerStack</t>
+  </si>
+  <si>
+    <t>施加几率</t>
+  </si>
+  <si>
+    <t>每层所需命中数</t>
   </si>
 </sst>
 </file>
@@ -577,10 +589,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -591,7 +603,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -634,8 +646,14 @@
       <c r="N2" t="s">
         <v>3</v>
       </c>
+      <c r="O2" t="s">
+        <v>8</v>
+      </c>
+      <c r="P2" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -678,8 +696,14 @@
       <c r="N3" t="s">
         <v>23</v>
       </c>
+      <c r="O3" t="s">
+        <v>62</v>
+      </c>
+      <c r="P3" t="s">
+        <v>63</v>
+      </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -722,8 +746,14 @@
       <c r="N4" t="s">
         <v>36</v>
       </c>
+      <c r="O4" t="s">
+        <v>64</v>
+      </c>
+      <c r="P4" t="s">
+        <v>65</v>
+      </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -746,7 +776,7 @@
         <v>1</v>
       </c>
       <c r="I5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -763,8 +793,14 @@
       <c r="N5" t="s">
         <v>41</v>
       </c>
+      <c r="O5">
+        <v>1</v>
+      </c>
+      <c r="P5">
+        <v>2</v>
+      </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
         <v>42</v>
       </c>
@@ -804,8 +840,14 @@
       <c r="N6" t="s">
         <v>41</v>
       </c>
+      <c r="O6">
+        <v>1</v>
+      </c>
+      <c r="P6">
+        <v>1</v>
+      </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -845,8 +887,14 @@
       <c r="N7" t="s">
         <v>41</v>
       </c>
+      <c r="O7">
+        <v>1</v>
+      </c>
+      <c r="P7">
+        <v>1</v>
+      </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A8" t="s">
         <v>50</v>
       </c>
@@ -886,8 +934,14 @@
       <c r="N8" t="s">
         <v>41</v>
       </c>
+      <c r="O8">
+        <v>1</v>
+      </c>
+      <c r="P8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -927,8 +981,14 @@
       <c r="N9" t="s">
         <v>41</v>
       </c>
+      <c r="O9">
+        <v>1</v>
+      </c>
+      <c r="P9">
+        <v>1</v>
+      </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A10" t="s">
         <v>58</v>
       </c>
@@ -951,7 +1011,7 @@
         <v>1</v>
       </c>
       <c r="I10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -967,6 +1027,12 @@
       </c>
       <c r="N10" t="s">
         <v>41</v>
+      </c>
+      <c r="O10">
+        <v>1</v>
+      </c>
+      <c r="P10">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>